<commit_message>
Aufgabe 3 fertig glaube ich
</commit_message>
<xml_diff>
--- a/GP2/Versuch_E17/Mitschriften_Versuch_E17.xlsx
+++ b/GP2/Versuch_E17/Mitschriften_Versuch_E17.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fynnlucca/Documents/Grundpraktikum-1/GP2/Versuch_E17/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C91B6736-E070-5C45-8799-2713DA160B58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEEF0EF4-B28C-3347-BD94-14B83EC1FF0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{D5C97754-4931-DE40-8915-B65B072F424C}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20400" xr2:uid="{D5C97754-4931-DE40-8915-B65B072F424C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -911,5 +911,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>